<commit_message>
modified:   analysis.ipynb     full -> nogeo data
</commit_message>
<xml_diff>
--- a/results/tab01.xlsx
+++ b/results/tab01.xlsx
@@ -476,8 +476,8 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5.125***
-[5.081, 5.168]</t>
+          <t>5.043***
+[4.996, 5.090]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -500,8 +500,8 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5.122***
-[5.078, 5.165]</t>
+          <t>5.038***
+[4.991, 5.085]</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -543,8 +543,8 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.205***
-[0.186, 0.223]</t>
+          <t>0.210***
+[0.189, 0.230]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -567,8 +567,8 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.205***
-[0.187, 0.224]</t>
+          <t>0.212***
+[0.191, 0.232]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R² = .01, R²adj = .01, F(1, 35480) = 469.53, p &lt; .0001, AIC = 106824.3, BIC = 106841.3, LL = -53410.1, MAE = 0.906, MAD = 0.924, N = 35481</t>
+          <t>R² = .01, R²adj = .01, F(1, 27563) = 402.20, p &lt; .0001, AIC = 80273.1, BIC = 80289.6, LL = -40134.6, MAE = 0.867, MAD = 0.879, N = 27564</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>R² = .01, R²adj = .01, F(1, 35480) = 477.06, p &lt; .0001, MAE = 0.906, MAD = 0.923, N = 35481</t>
+          <t>R² = .01, R²adj = .01, F(1, 27563) = 412.13, p &lt; .0001, MAE = 0.867, MAD = 0.878, N = 27564</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">

</xml_diff>